<commit_message>
Fixed code and parameter-study-2 sheet from 7-14.
</commit_message>
<xml_diff>
--- a/Results/results_7-14(gaussian)/rbf_fd_parameter_study_2.xlsx
+++ b/Results/results_7-14(gaussian)/rbf_fd_parameter_study_2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zeonv\Documents\Projects\RBF-FD-Elliptic\Results\results_7-14(gaussian)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Users\zeonv\Documents\Projects\RBF-FD-Elliptic\Results\results_7-14(gaussian)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D414C19D-9815-4913-9FF5-649E7AFE0184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A779E0-E0CE-4E28-B19A-4CCE155BEFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="21">
   <si>
     <t>Nx</t>
   </si>
@@ -1020,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -1868,801 +1868,6 @@
         <v>18</v>
       </c>
       <c r="Q16">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>500</v>
-      </c>
-      <c r="B17">
-        <v>500</v>
-      </c>
-      <c r="C17">
-        <v>0.05</v>
-      </c>
-      <c r="D17">
-        <v>5</v>
-      </c>
-      <c r="E17">
-        <v>5</v>
-      </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="G17">
-        <v>1E-3</v>
-      </c>
-      <c r="H17">
-        <v>12</v>
-      </c>
-      <c r="I17" t="b">
-        <v>0</v>
-      </c>
-      <c r="J17" t="b">
-        <v>1</v>
-      </c>
-      <c r="K17">
-        <v>4212.3268772723377</v>
-      </c>
-      <c r="L17">
-        <v>2795.779531038314</v>
-      </c>
-      <c r="M17">
-        <v>5942.355564831777</v>
-      </c>
-      <c r="N17">
-        <v>0.99972055757785361</v>
-      </c>
-      <c r="O17">
-        <v>0.99972058247323869</v>
-      </c>
-      <c r="P17" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q17">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>500</v>
-      </c>
-      <c r="B18">
-        <v>500</v>
-      </c>
-      <c r="C18">
-        <v>0.1</v>
-      </c>
-      <c r="D18">
-        <v>5</v>
-      </c>
-      <c r="E18">
-        <v>5</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-      <c r="G18">
-        <v>1E-3</v>
-      </c>
-      <c r="H18">
-        <v>12</v>
-      </c>
-      <c r="I18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J18" t="b">
-        <v>1</v>
-      </c>
-      <c r="K18">
-        <v>1052.19863885718</v>
-      </c>
-      <c r="L18">
-        <v>698.35903138868071</v>
-      </c>
-      <c r="M18">
-        <v>1485.1374891298351</v>
-      </c>
-      <c r="N18">
-        <v>0.9988822303044389</v>
-      </c>
-      <c r="O18">
-        <v>0.99888262896482938</v>
-      </c>
-      <c r="P18" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q18">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>500</v>
-      </c>
-      <c r="B19">
-        <v>500</v>
-      </c>
-      <c r="C19">
-        <v>0.5</v>
-      </c>
-      <c r="D19">
-        <v>5</v>
-      </c>
-      <c r="E19">
-        <v>5</v>
-      </c>
-      <c r="F19">
-        <v>1</v>
-      </c>
-      <c r="G19">
-        <v>1E-3</v>
-      </c>
-      <c r="H19">
-        <v>12</v>
-      </c>
-      <c r="I19" t="b">
-        <v>0</v>
-      </c>
-      <c r="J19" t="b">
-        <v>1</v>
-      </c>
-      <c r="K19">
-        <v>1.231147864098138E-4</v>
-      </c>
-      <c r="L19">
-        <v>1.150312817627645E-4</v>
-      </c>
-      <c r="M19">
-        <v>1.098005132761358E-4</v>
-      </c>
-      <c r="N19">
-        <v>6.0278497470036059E-5</v>
-      </c>
-      <c r="O19">
-        <v>8.2131147281380089E-5</v>
-      </c>
-      <c r="P19" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q19">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>500</v>
-      </c>
-      <c r="B20">
-        <v>500</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
-        <v>5</v>
-      </c>
-      <c r="E20">
-        <v>5</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20">
-        <v>1E-3</v>
-      </c>
-      <c r="H20">
-        <v>12</v>
-      </c>
-      <c r="I20" t="b">
-        <v>0</v>
-      </c>
-      <c r="J20" t="b">
-        <v>1</v>
-      </c>
-      <c r="K20">
-        <v>8.7866498645472073E-6</v>
-      </c>
-      <c r="L20">
-        <v>5.2825900807237283E-6</v>
-      </c>
-      <c r="M20">
-        <v>9.1736655971593197E-6</v>
-      </c>
-      <c r="N20">
-        <v>1.430033557997225E-5</v>
-      </c>
-      <c r="O20">
-        <v>1.8403051746201768E-5</v>
-      </c>
-      <c r="P20" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>500</v>
-      </c>
-      <c r="B21">
-        <v>500</v>
-      </c>
-      <c r="C21">
-        <v>2</v>
-      </c>
-      <c r="D21">
-        <v>5</v>
-      </c>
-      <c r="E21">
-        <v>5</v>
-      </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
-      <c r="G21">
-        <v>1E-3</v>
-      </c>
-      <c r="H21">
-        <v>12</v>
-      </c>
-      <c r="I21" t="b">
-        <v>0</v>
-      </c>
-      <c r="J21" t="b">
-        <v>1</v>
-      </c>
-      <c r="K21">
-        <v>4.5480754005138426E-6</v>
-      </c>
-      <c r="L21">
-        <v>3.7939462585287138E-6</v>
-      </c>
-      <c r="M21">
-        <v>5.6644997656443223E-6</v>
-      </c>
-      <c r="N21">
-        <v>8.168635047016511E-6</v>
-      </c>
-      <c r="O21">
-        <v>1.0583031570442759E-5</v>
-      </c>
-      <c r="P21" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>500</v>
-      </c>
-      <c r="B22">
-        <v>500</v>
-      </c>
-      <c r="C22">
-        <v>2.5</v>
-      </c>
-      <c r="D22">
-        <v>5</v>
-      </c>
-      <c r="E22">
-        <v>5</v>
-      </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22">
-        <v>1E-3</v>
-      </c>
-      <c r="H22">
-        <v>12</v>
-      </c>
-      <c r="I22" t="b">
-        <v>0</v>
-      </c>
-      <c r="J22" t="b">
-        <v>1</v>
-      </c>
-      <c r="K22">
-        <v>5.9883294357672366E-6</v>
-      </c>
-      <c r="L22">
-        <v>5.3115661048053572E-6</v>
-      </c>
-      <c r="M22">
-        <v>5.4164205982864359E-6</v>
-      </c>
-      <c r="N22">
-        <v>4.610566224304919E-6</v>
-      </c>
-      <c r="O22">
-        <v>5.8667355935049341E-6</v>
-      </c>
-      <c r="P22" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q22">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>500</v>
-      </c>
-      <c r="B23">
-        <v>500</v>
-      </c>
-      <c r="C23">
-        <v>3</v>
-      </c>
-      <c r="D23">
-        <v>5</v>
-      </c>
-      <c r="E23">
-        <v>5</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>1E-3</v>
-      </c>
-      <c r="H23">
-        <v>12</v>
-      </c>
-      <c r="I23" t="b">
-        <v>0</v>
-      </c>
-      <c r="J23" t="b">
-        <v>1</v>
-      </c>
-      <c r="K23">
-        <v>4.4633991824626258E-7</v>
-      </c>
-      <c r="L23">
-        <v>3.737447598599238E-7</v>
-      </c>
-      <c r="M23">
-        <v>8.8921374335931358E-7</v>
-      </c>
-      <c r="N23">
-        <v>1.4191535409136751E-6</v>
-      </c>
-      <c r="O23">
-        <v>1.9316734334396412E-6</v>
-      </c>
-      <c r="P23" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q23">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>500</v>
-      </c>
-      <c r="B24">
-        <v>500</v>
-      </c>
-      <c r="C24">
-        <v>3.5</v>
-      </c>
-      <c r="D24">
-        <v>5</v>
-      </c>
-      <c r="E24">
-        <v>5</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24">
-        <v>1E-3</v>
-      </c>
-      <c r="H24">
-        <v>12</v>
-      </c>
-      <c r="I24" t="b">
-        <v>0</v>
-      </c>
-      <c r="J24" t="b">
-        <v>1</v>
-      </c>
-      <c r="K24">
-        <v>1.6582551924604369E-5</v>
-      </c>
-      <c r="L24">
-        <v>1.4922256565332849E-5</v>
-      </c>
-      <c r="M24">
-        <v>1.4726377413215059E-5</v>
-      </c>
-      <c r="N24">
-        <v>1.083270754859958E-5</v>
-      </c>
-      <c r="O24">
-        <v>1.3806963070273689E-5</v>
-      </c>
-      <c r="P24" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q24">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>500</v>
-      </c>
-      <c r="B25">
-        <v>500</v>
-      </c>
-      <c r="C25">
-        <v>4</v>
-      </c>
-      <c r="D25">
-        <v>5</v>
-      </c>
-      <c r="E25">
-        <v>5</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
-        <v>1E-3</v>
-      </c>
-      <c r="H25">
-        <v>12</v>
-      </c>
-      <c r="I25" t="b">
-        <v>0</v>
-      </c>
-      <c r="J25" t="b">
-        <v>1</v>
-      </c>
-      <c r="K25">
-        <v>4.6096548457771861E-5</v>
-      </c>
-      <c r="L25">
-        <v>4.2069444378068183E-5</v>
-      </c>
-      <c r="M25">
-        <v>4.0716553879546551E-5</v>
-      </c>
-      <c r="N25">
-        <v>2.7068064391597271E-5</v>
-      </c>
-      <c r="O25">
-        <v>3.3939202233137857E-5</v>
-      </c>
-      <c r="P25" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>500</v>
-      </c>
-      <c r="B26">
-        <v>500</v>
-      </c>
-      <c r="C26">
-        <v>5</v>
-      </c>
-      <c r="D26">
-        <v>5</v>
-      </c>
-      <c r="E26">
-        <v>5</v>
-      </c>
-      <c r="F26">
-        <v>1</v>
-      </c>
-      <c r="G26">
-        <v>1E-3</v>
-      </c>
-      <c r="H26">
-        <v>12</v>
-      </c>
-      <c r="I26" t="b">
-        <v>0</v>
-      </c>
-      <c r="J26" t="b">
-        <v>1</v>
-      </c>
-      <c r="K26">
-        <v>1.6579240760040449E-4</v>
-      </c>
-      <c r="L26">
-        <v>1.5333400505314991E-4</v>
-      </c>
-      <c r="M26">
-        <v>1.4685215686450391E-4</v>
-      </c>
-      <c r="N26">
-        <v>8.7851020560272502E-5</v>
-      </c>
-      <c r="O26">
-        <v>1.1301759222454471E-4</v>
-      </c>
-      <c r="P26" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q26">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>500</v>
-      </c>
-      <c r="B27">
-        <v>500</v>
-      </c>
-      <c r="C27">
-        <v>7.5</v>
-      </c>
-      <c r="D27">
-        <v>5</v>
-      </c>
-      <c r="E27">
-        <v>5</v>
-      </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27">
-        <v>1E-3</v>
-      </c>
-      <c r="H27">
-        <v>12</v>
-      </c>
-      <c r="I27" t="b">
-        <v>0</v>
-      </c>
-      <c r="J27" t="b">
-        <v>1</v>
-      </c>
-      <c r="K27">
-        <v>1.1121754007251919E-3</v>
-      </c>
-      <c r="L27">
-        <v>1.0409954131288849E-3</v>
-      </c>
-      <c r="M27">
-        <v>9.934489969662581E-4</v>
-      </c>
-      <c r="N27">
-        <v>5.364260902599588E-4</v>
-      </c>
-      <c r="O27">
-        <v>7.4085246523665732E-4</v>
-      </c>
-      <c r="P27" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q27">
-        <v>7.5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>500</v>
-      </c>
-      <c r="B28">
-        <v>500</v>
-      </c>
-      <c r="C28">
-        <v>10</v>
-      </c>
-      <c r="D28">
-        <v>5</v>
-      </c>
-      <c r="E28">
-        <v>5</v>
-      </c>
-      <c r="F28">
-        <v>1</v>
-      </c>
-      <c r="G28">
-        <v>1E-3</v>
-      </c>
-      <c r="H28">
-        <v>12</v>
-      </c>
-      <c r="I28" t="b">
-        <v>0</v>
-      </c>
-      <c r="J28" t="b">
-        <v>1</v>
-      </c>
-      <c r="K28">
-        <v>3.844730649185816E-3</v>
-      </c>
-      <c r="L28">
-        <v>3.5998967085132602E-3</v>
-      </c>
-      <c r="M28">
-        <v>3.4351275598339041E-3</v>
-      </c>
-      <c r="N28">
-        <v>1.8446489017349659E-3</v>
-      </c>
-      <c r="O28">
-        <v>2.5528278429827992E-3</v>
-      </c>
-      <c r="P28" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q28">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>500</v>
-      </c>
-      <c r="B29">
-        <v>500</v>
-      </c>
-      <c r="C29">
-        <v>15</v>
-      </c>
-      <c r="D29">
-        <v>5</v>
-      </c>
-      <c r="E29">
-        <v>5</v>
-      </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
-      <c r="G29">
-        <v>1E-3</v>
-      </c>
-      <c r="H29">
-        <v>12</v>
-      </c>
-      <c r="I29" t="b">
-        <v>0</v>
-      </c>
-      <c r="J29" t="b">
-        <v>1</v>
-      </c>
-      <c r="K29">
-        <v>2.1086886366514321E-2</v>
-      </c>
-      <c r="L29">
-        <v>1.963672496993394E-2</v>
-      </c>
-      <c r="M29">
-        <v>1.874221505450752E-2</v>
-      </c>
-      <c r="N29">
-        <v>1.039066645838637E-2</v>
-      </c>
-      <c r="O29">
-        <v>1.373704241515422E-2</v>
-      </c>
-      <c r="P29" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q29">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>500</v>
-      </c>
-      <c r="B30">
-        <v>500</v>
-      </c>
-      <c r="C30">
-        <v>20</v>
-      </c>
-      <c r="D30">
-        <v>5</v>
-      </c>
-      <c r="E30">
-        <v>5</v>
-      </c>
-      <c r="F30">
-        <v>1</v>
-      </c>
-      <c r="G30">
-        <v>1E-3</v>
-      </c>
-      <c r="H30">
-        <v>12</v>
-      </c>
-      <c r="I30" t="b">
-        <v>0</v>
-      </c>
-      <c r="J30" t="b">
-        <v>1</v>
-      </c>
-      <c r="K30">
-        <v>7.1204690297052897E-2</v>
-      </c>
-      <c r="L30">
-        <v>6.6208979443173707E-2</v>
-      </c>
-      <c r="M30">
-        <v>6.3199610309219847E-2</v>
-      </c>
-      <c r="N30">
-        <v>3.4037448892087013E-2</v>
-      </c>
-      <c r="O30">
-        <v>4.434371288840832E-2</v>
-      </c>
-      <c r="P30" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q30">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>500</v>
-      </c>
-      <c r="B31">
-        <v>500</v>
-      </c>
-      <c r="C31">
-        <v>30</v>
-      </c>
-      <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="E31">
-        <v>5</v>
-      </c>
-      <c r="F31">
-        <v>1</v>
-      </c>
-      <c r="G31">
-        <v>1E-3</v>
-      </c>
-      <c r="H31">
-        <v>12</v>
-      </c>
-      <c r="I31" t="b">
-        <v>0</v>
-      </c>
-      <c r="J31" t="b">
-        <v>1</v>
-      </c>
-      <c r="K31">
-        <v>0.50343241926640914</v>
-      </c>
-      <c r="L31">
-        <v>0.46877894332005232</v>
-      </c>
-      <c r="M31">
-        <v>0.4474266713697132</v>
-      </c>
-      <c r="N31">
-        <v>0.17664293877167639</v>
-      </c>
-      <c r="O31">
-        <v>0.22781900137290981</v>
-      </c>
-      <c r="P31" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q31">
         <v>30</v>
       </c>
     </row>

</xml_diff>